<commit_message>
feat: add dqn model
</commit_message>
<xml_diff>
--- a/CCTV Data Remastered.xlsx
+++ b/CCTV Data Remastered.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Kuliah\Skripsi\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Kuliah\Skripsi\Project\SUMO-dinamic-tuning-AI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5116FFD-3A7C-4484-AF86-1A866B418F3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{559AF5DD-A8C5-45E9-8D20-68D703D6F1A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F9AC95A1-0791-4863-B684-AC15BB9D8B18}"/>
   </bookViews>
@@ -708,10 +708,18 @@
       <c r="D4" s="2">
         <v>57</v>
       </c>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
+      <c r="E4" s="2">
+        <v>64</v>
+      </c>
+      <c r="F4" s="2">
+        <v>6</v>
+      </c>
+      <c r="G4" s="2">
+        <v>88</v>
+      </c>
+      <c r="H4" s="2">
+        <v>71</v>
+      </c>
       <c r="I4" s="2">
         <f t="shared" ref="I4:I30" si="1">C4*6</f>
         <v>780</v>
@@ -722,19 +730,19 @@
       </c>
       <c r="K4" s="2">
         <f t="shared" ref="K4:K30" si="3">E4*6</f>
-        <v>0</v>
+        <v>384</v>
       </c>
       <c r="L4" s="2">
         <f t="shared" ref="L4:L30" si="4">F4*6</f>
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="M4" s="2">
         <f t="shared" ref="M4:M30" si="5">G4*6</f>
-        <v>0</v>
+        <v>528</v>
       </c>
       <c r="N4" s="2">
         <f t="shared" ref="N4:N30" si="6">H4*6</f>
-        <v>0</v>
+        <v>426</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">

</xml_diff>